<commit_message>
Correcation to VAT rate
</commit_message>
<xml_diff>
--- a/InputData/io-model/VoSTR/VAT or Sales Tax Rate.xlsx
+++ b/InputData/io-model/VoSTR/VAT or Sales Tax Rate.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\kjh_local\NEXTgroup_local\2025_local\2. EPS\업데이트 파일\eps-southkorea-3.3.1_2025update_v4.0.3\InputData\io-model\VoSTR\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mary Francis Swint\Vensim\eps-southkorea\InputData\io-model\VoSTR\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAEAF1E4-1970-45EE-8027-49FC40CD2B68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BBFD46D-B478-4601-BCF6-9A91A331CC74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-36240" yWindow="-2490" windowWidth="28800" windowHeight="15225" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -493,14 +493,14 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="176" formatCode="0.0000"/>
-    <numFmt numFmtId="177" formatCode="#,##0.0#"/>
+    <numFmt numFmtId="164" formatCode="0.0000"/>
+    <numFmt numFmtId="165" formatCode="#,##0.0#"/>
   </numFmts>
   <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -508,7 +508,7 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -516,13 +516,13 @@
       <i/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="8"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="129"/>
       <scheme val="minor"/>
@@ -531,7 +531,7 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -731,7 +731,7 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -753,7 +753,7 @@
     <xf numFmtId="3" fontId="7" fillId="4" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="7" fillId="4" borderId="6" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="7" fillId="4" borderId="6" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="7" fillId="5" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -765,7 +765,7 @@
     <xf numFmtId="3" fontId="7" fillId="5" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="7" fillId="5" borderId="6" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="7" fillId="5" borderId="6" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="7" fillId="5" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -777,7 +777,7 @@
     <xf numFmtId="3" fontId="7" fillId="5" borderId="8" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="7" fillId="5" borderId="9" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="7" fillId="5" borderId="9" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1">
@@ -786,12 +786,12 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="176" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="3">
-    <cellStyle name="표준" xfId="0" builtinId="0"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="표준 2" xfId="2" xr:uid="{7A8253D2-D3BA-44D0-BA2D-8B474419AA43}"/>
-    <cellStyle name="하이퍼링크" xfId="1" builtinId="8"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1094,7 +1094,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G18"/>
-  <sheetFormatPr defaultRowHeight="16.5"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
@@ -1198,11 +1198,11 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{40D66251-3A42-4ADF-A485-C8536302A941}">
   <dimension ref="A1:H43"/>
-  <sheetFormatPr defaultRowHeight="12.75"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="12.5"/>
   <cols>
     <col min="1" max="2" width="9" style="10"/>
-    <col min="3" max="7" width="21.625" style="10" customWidth="1"/>
-    <col min="8" max="8" width="17.375" style="10" customWidth="1"/>
+    <col min="3" max="7" width="21.6328125" style="10" customWidth="1"/>
+    <col min="8" max="8" width="17.36328125" style="10" customWidth="1"/>
     <col min="9" max="16384" width="9" style="10"/>
   </cols>
   <sheetData>
@@ -2336,13 +2336,13 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AQ2"/>
-  <sheetFormatPr defaultRowHeight="16.5"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="15.5" customWidth="1"/>
-    <col min="2" max="2" width="26.25" customWidth="1"/>
+    <col min="1" max="1" width="15.453125" customWidth="1"/>
+    <col min="2" max="2" width="26.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:43" ht="33">
+    <row r="1" spans="1:43" ht="29">
       <c r="A1" s="3" t="s">
         <v>44</v>
       </c>
@@ -2478,115 +2478,115 @@
         <v>147</v>
       </c>
       <c r="B2" s="6">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="C2" s="6">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="D2" s="6">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="E2" s="6">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="F2" s="6">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="G2" s="6">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="H2" s="6">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="I2" s="6">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="J2" s="6">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="K2" s="6">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="L2" s="6">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="M2" s="6">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="N2" s="6">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="O2" s="6">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="P2" s="6">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="Q2" s="6">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="R2" s="6">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="S2" s="6">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="T2" s="6">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="U2" s="6">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="V2" s="6">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="W2" s="6">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="X2" s="6">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="Y2" s="6">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="Z2" s="6">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="AA2" s="6">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="AB2" s="6">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="AC2" s="6">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="AD2" s="6">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="AE2" s="6">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="AF2" s="6">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="AG2" s="6">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="AH2" s="6">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="AI2" s="6">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="AJ2" s="6">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="AK2" s="6">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="AL2" s="6">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="AM2" s="25">
         <v>0</v>
@@ -2595,13 +2595,13 @@
         <v>0</v>
       </c>
       <c r="AO2" s="6">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="AP2" s="6">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="AQ2" s="6">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
     </row>
   </sheetData>
@@ -2756,6 +2756,12 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -2764,20 +2770,37 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{755676E5-16DF-4B5A-9AAD-AD7FD0EED4C8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{755676E5-16DF-4B5A-9AAD-AD7FD0EED4C8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="40f4d404-d193-41dc-bb72-733c1e774208"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4A3602F7-CDEC-4992-817A-78EE06933531}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8510F28C-B720-441A-AAC0-46281F3CEBA6}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8510F28C-B720-441A-AAC0-46281F3CEBA6}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4A3602F7-CDEC-4992-817A-78EE06933531}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>